<commit_message>
Add WNBA 2025 cash tab to Spotrac payroll workbook
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PFAktiXyafs53JJMEMzshM
</commit_message>
<xml_diff>
--- a/reports/Spotrac team payrolls.xlsx
+++ b/reports/Spotrac team payrolls.xlsx
@@ -14,6 +14,7 @@
     <sheet name="MLB" sheetId="4" state="visible" r:id="rId6"/>
     <sheet name="NHL" sheetId="5" state="visible" r:id="rId7"/>
     <sheet name="MLS" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="WNBA" sheetId="7" state="visible" r:id="rId9"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="358" uniqueCount="220">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="392" uniqueCount="228">
   <si>
     <t xml:space="preserve">Spotrac team payroll tables transcribed from five screenshots supplied by the user (transcribed Oct 21, 2026).</t>
   </si>
@@ -45,6 +46,9 @@
     <t xml:space="preserve">NHL | Spotrac NHL cash tracker | Not shown; records match 2025-26 | Cash paid: Active + Dead + other. Screenshot had no totals row; totals here are SUM formulas.</t>
   </si>
   <si>
+    <t xml:space="preserve">WNBA | Spotrac WNBA cash tracker | 2025 (shown in screenshot) | Cash paid: Active + Dead + other</t>
+  </si>
+  <si>
     <t xml:space="preserve">MLS | Spotrac MLS cap tracker | Not shown; likely 2026 | Cap allocation (not cash): Total Allocation = Senior + Supplemental + Dead. Row 31 'MLS' is league-held dead money.</t>
   </si>
   <si>
@@ -685,6 +689,27 @@
   </si>
   <si>
     <t xml:space="preserve">Spotrac's screenshot showed only an Averages row (no Totals); Totals here are computed.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WNBA 2025 team cash payroll (Spotrac)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Playoff team</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Champion</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CON</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spotrac's Record column showed only icons (star = playoff team, trophy = champion); those are written as text here.</t>
   </si>
 </sst>
 </file>
@@ -1135,7 +1160,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:A15"/>
+  <dimension ref="A1:A16"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="150"/>
@@ -1180,12 +1205,12 @@
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="2"/>
+      <c r="A9" s="2" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="1" t="s">
-        <v>7</v>
-      </c>
+      <c r="A10" s="1"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
@@ -1210,6 +1235,11 @@
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
         <v>12</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="2" t="s">
+        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -1241,33 +1271,33 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1275,10 +1305,10 @@
         <v>1</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D4" s="5" t="n">
         <v>53</v>
@@ -1301,10 +1331,10 @@
         <v>2</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D5" s="5" t="n">
         <v>53</v>
@@ -1327,10 +1357,10 @@
         <v>3</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D6" s="5" t="n">
         <v>54</v>
@@ -1353,10 +1383,10 @@
         <v>4</v>
       </c>
       <c r="B7" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C7" s="2" t="s">
         <v>28</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>27</v>
       </c>
       <c r="D7" s="5" t="n">
         <v>52</v>
@@ -1379,10 +1409,10 @@
         <v>5</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D8" s="5" t="n">
         <v>52</v>
@@ -1405,10 +1435,10 @@
         <v>6</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D9" s="5" t="n">
         <v>52</v>
@@ -1431,10 +1461,10 @@
         <v>7</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D10" s="5" t="n">
         <v>52</v>
@@ -1457,10 +1487,10 @@
         <v>8</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D11" s="5" t="n">
         <v>53</v>
@@ -1483,10 +1513,10 @@
         <v>9</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D12" s="5" t="n">
         <v>53</v>
@@ -1509,10 +1539,10 @@
         <v>10</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D13" s="5" t="n">
         <v>53</v>
@@ -1535,10 +1565,10 @@
         <v>11</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D14" s="5" t="n">
         <v>52</v>
@@ -1561,10 +1591,10 @@
         <v>12</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D15" s="5" t="n">
         <v>53</v>
@@ -1587,10 +1617,10 @@
         <v>13</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D16" s="5" t="n">
         <v>51</v>
@@ -1613,10 +1643,10 @@
         <v>14</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D17" s="5" t="n">
         <v>53</v>
@@ -1639,10 +1669,10 @@
         <v>15</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D18" s="5" t="n">
         <v>52</v>
@@ -1665,10 +1695,10 @@
         <v>16</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D19" s="5" t="n">
         <v>54</v>
@@ -1691,10 +1721,10 @@
         <v>17</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D20" s="5" t="n">
         <v>53</v>
@@ -1717,10 +1747,10 @@
         <v>18</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D21" s="5" t="n">
         <v>53</v>
@@ -1743,10 +1773,10 @@
         <v>19</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D22" s="5" t="n">
         <v>52</v>
@@ -1769,10 +1799,10 @@
         <v>20</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D23" s="5" t="n">
         <v>52</v>
@@ -1795,10 +1825,10 @@
         <v>21</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D24" s="5" t="n">
         <v>53</v>
@@ -1821,10 +1851,10 @@
         <v>22</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D25" s="5" t="n">
         <v>53</v>
@@ -1847,10 +1877,10 @@
         <v>23</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D26" s="5" t="n">
         <v>53</v>
@@ -1873,10 +1903,10 @@
         <v>24</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D27" s="5" t="n">
         <v>52</v>
@@ -1899,10 +1929,10 @@
         <v>25</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D28" s="5" t="n">
         <v>53</v>
@@ -1925,10 +1955,10 @@
         <v>26</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D29" s="5" t="n">
         <v>53</v>
@@ -1951,10 +1981,10 @@
         <v>27</v>
       </c>
       <c r="B30" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="C30" s="2" t="s">
         <v>62</v>
-      </c>
-      <c r="C30" s="2" t="s">
-        <v>61</v>
       </c>
       <c r="D30" s="5" t="n">
         <v>52</v>
@@ -1977,10 +2007,10 @@
         <v>28</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D31" s="5" t="n">
         <v>53</v>
@@ -2003,10 +2033,10 @@
         <v>29</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D32" s="5" t="n">
         <v>52</v>
@@ -2029,10 +2059,10 @@
         <v>30</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D33" s="5" t="n">
         <v>52</v>
@@ -2055,10 +2085,10 @@
         <v>31</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D34" s="5" t="n">
         <v>53</v>
@@ -2081,10 +2111,10 @@
         <v>32</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D35" s="5" t="n">
         <v>53</v>
@@ -2104,7 +2134,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="8" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B36" s="9"/>
       <c r="C36" s="9"/>
@@ -2128,7 +2158,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="8" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B37" s="9"/>
       <c r="C37" s="9"/>
@@ -2155,7 +2185,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="13" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D38" s="14" t="n">
         <v>1684</v>
@@ -2172,7 +2202,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="13" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D39" s="14" t="n">
         <f aca="false">D36-D38</f>
@@ -2220,36 +2250,36 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="I3" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2257,10 +2287,10 @@
         <v>28</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D4" s="5" t="n">
         <v>15</v>
@@ -2286,10 +2316,10 @@
         <v>15</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D5" s="5" t="n">
         <v>15</v>
@@ -2315,10 +2345,10 @@
         <v>1</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D6" s="5" t="n">
         <v>15</v>
@@ -2344,10 +2374,10 @@
         <v>2</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D7" s="5" t="n">
         <v>15</v>
@@ -2373,10 +2403,10 @@
         <v>8</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D8" s="5" t="n">
         <v>15</v>
@@ -2402,10 +2432,10 @@
         <v>23</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D9" s="5" t="n">
         <v>15</v>
@@ -2431,10 +2461,10 @@
         <v>26</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D10" s="5" t="n">
         <v>15</v>
@@ -2460,10 +2490,10 @@
         <v>10</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D11" s="5" t="n">
         <v>15</v>
@@ -2489,10 +2519,10 @@
         <v>4</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D12" s="5" t="n">
         <v>15</v>
@@ -2518,10 +2548,10 @@
         <v>16</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D13" s="5" t="n">
         <v>15</v>
@@ -2547,10 +2577,10 @@
         <v>5</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D14" s="5" t="n">
         <v>15</v>
@@ -2576,10 +2606,10 @@
         <v>22</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D15" s="5" t="n">
         <v>15</v>
@@ -2605,10 +2635,10 @@
         <v>29</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D16" s="5" t="n">
         <v>15</v>
@@ -2634,10 +2664,10 @@
         <v>7</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D17" s="5" t="n">
         <v>15</v>
@@ -2663,10 +2693,10 @@
         <v>25</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D18" s="5" t="n">
         <v>15</v>
@@ -2692,10 +2722,10 @@
         <v>6</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D19" s="5" t="n">
         <v>15</v>
@@ -2721,10 +2751,10 @@
         <v>11</v>
       </c>
       <c r="B20" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="C20" s="2" t="s">
         <v>95</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>94</v>
       </c>
       <c r="D20" s="5" t="n">
         <v>15</v>
@@ -2750,10 +2780,10 @@
         <v>14</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D21" s="5" t="n">
         <v>15</v>
@@ -2779,10 +2809,10 @@
         <v>13</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D22" s="5" t="n">
         <v>15</v>
@@ -2808,10 +2838,10 @@
         <v>19</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D23" s="5" t="n">
         <v>15</v>
@@ -2837,10 +2867,10 @@
         <v>24</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D24" s="5" t="n">
         <v>15</v>
@@ -2866,10 +2896,10 @@
         <v>3</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D25" s="5" t="n">
         <v>15</v>
@@ -2895,10 +2925,10 @@
         <v>20</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D26" s="5" t="n">
         <v>15</v>
@@ -2924,10 +2954,10 @@
         <v>27</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D27" s="5" t="n">
         <v>15</v>
@@ -2953,10 +2983,10 @@
         <v>12</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D28" s="5" t="n">
         <v>15</v>
@@ -2982,10 +3012,10 @@
         <v>17</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D29" s="5" t="n">
         <v>15</v>
@@ -3011,10 +3041,10 @@
         <v>9</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D30" s="5" t="n">
         <v>15</v>
@@ -3040,10 +3070,10 @@
         <v>18</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D31" s="5" t="n">
         <v>15</v>
@@ -3069,10 +3099,10 @@
         <v>30</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D32" s="5" t="n">
         <v>15</v>
@@ -3098,10 +3128,10 @@
         <v>21</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D33" s="5" t="n">
         <v>15</v>
@@ -3124,7 +3154,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="8" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B34" s="9"/>
       <c r="C34" s="9"/>
@@ -3152,7 +3182,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="8" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B35" s="9"/>
       <c r="C35" s="9"/>
@@ -3183,7 +3213,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="13" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D36" s="14" t="n">
         <v>450</v>
@@ -3203,7 +3233,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="13" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D37" s="14" t="n">
         <f aca="false">D34-D36</f>
@@ -3255,33 +3285,33 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3289,10 +3319,10 @@
         <v>1</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D4" s="5" t="n">
         <v>28</v>
@@ -3315,10 +3345,10 @@
         <v>2</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D5" s="5" t="n">
         <v>27</v>
@@ -3341,10 +3371,10 @@
         <v>3</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D6" s="5" t="n">
         <v>28</v>
@@ -3367,10 +3397,10 @@
         <v>4</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D7" s="5" t="n">
         <v>27</v>
@@ -3393,10 +3423,10 @@
         <v>5</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D8" s="5" t="n">
         <v>28</v>
@@ -3419,10 +3449,10 @@
         <v>6</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D9" s="5" t="n">
         <v>28</v>
@@ -3445,10 +3475,10 @@
         <v>7</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D10" s="5" t="n">
         <v>32</v>
@@ -3471,10 +3501,10 @@
         <v>8</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D11" s="5" t="n">
         <v>28</v>
@@ -3497,10 +3527,10 @@
         <v>9</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D12" s="5" t="n">
         <v>28</v>
@@ -3523,10 +3553,10 @@
         <v>10</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D13" s="5" t="n">
         <v>28</v>
@@ -3549,10 +3579,10 @@
         <v>11</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D14" s="5" t="n">
         <v>28</v>
@@ -3575,10 +3605,10 @@
         <v>12</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D15" s="5" t="n">
         <v>28</v>
@@ -3601,10 +3631,10 @@
         <v>13</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D16" s="5" t="n">
         <v>28</v>
@@ -3627,10 +3657,10 @@
         <v>14</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D17" s="5" t="n">
         <v>28</v>
@@ -3653,10 +3683,10 @@
         <v>15</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D18" s="5" t="n">
         <v>28</v>
@@ -3679,10 +3709,10 @@
         <v>16</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D19" s="5" t="n">
         <v>28</v>
@@ -3705,10 +3735,10 @@
         <v>17</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D20" s="5" t="n">
         <v>28</v>
@@ -3731,10 +3761,10 @@
         <v>18</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D21" s="5" t="n">
         <v>28</v>
@@ -3757,10 +3787,10 @@
         <v>19</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D22" s="5" t="n">
         <v>28</v>
@@ -3783,10 +3813,10 @@
         <v>20</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="D23" s="5" t="n">
         <v>28</v>
@@ -3809,10 +3839,10 @@
         <v>21</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="D24" s="5" t="n">
         <v>28</v>
@@ -3835,10 +3865,10 @@
         <v>22</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D25" s="5" t="n">
         <v>28</v>
@@ -3861,10 +3891,10 @@
         <v>23</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D26" s="5" t="n">
         <v>28</v>
@@ -3887,10 +3917,10 @@
         <v>24</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D27" s="5" t="n">
         <v>28</v>
@@ -3913,10 +3943,10 @@
         <v>25</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D28" s="5" t="n">
         <v>28</v>
@@ -3939,10 +3969,10 @@
         <v>26</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D29" s="5" t="n">
         <v>28</v>
@@ -3965,10 +3995,10 @@
         <v>27</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D30" s="5" t="n">
         <v>31</v>
@@ -3991,10 +4021,10 @@
         <v>28</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D31" s="5" t="n">
         <v>28</v>
@@ -4017,10 +4047,10 @@
         <v>29</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D32" s="5" t="n">
         <v>28</v>
@@ -4043,10 +4073,10 @@
         <v>30</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="D33" s="5" t="n">
         <v>28</v>
@@ -4066,7 +4096,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="8" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B34" s="9"/>
       <c r="C34" s="9"/>
@@ -4090,7 +4120,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="8" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B35" s="9"/>
       <c r="C35" s="9"/>
@@ -4117,7 +4147,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="13" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D36" s="14" t="n">
         <v>845</v>
@@ -4134,7 +4164,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="13" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D37" s="14" t="n">
         <f aca="false">D34-D36</f>
@@ -4182,33 +4212,33 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4216,10 +4246,10 @@
         <v>1</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D4" s="5" t="n">
         <v>23</v>
@@ -4242,10 +4272,10 @@
         <v>2</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="D5" s="5" t="n">
         <v>27</v>
@@ -4268,10 +4298,10 @@
         <v>3</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D6" s="5" t="n">
         <v>24</v>
@@ -4294,10 +4324,10 @@
         <v>4</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D7" s="5" t="n">
         <v>25</v>
@@ -4320,10 +4350,10 @@
         <v>5</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="D8" s="5" t="n">
         <v>22</v>
@@ -4346,10 +4376,10 @@
         <v>6</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="D9" s="5" t="n">
         <v>26</v>
@@ -4372,10 +4402,10 @@
         <v>7</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="D10" s="5" t="n">
         <v>23</v>
@@ -4398,10 +4428,10 @@
         <v>8</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="D11" s="5" t="n">
         <v>26</v>
@@ -4424,10 +4454,10 @@
         <v>9</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D12" s="5" t="n">
         <v>26</v>
@@ -4450,10 +4480,10 @@
         <v>10</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="D13" s="5" t="n">
         <v>25</v>
@@ -4476,10 +4506,10 @@
         <v>11</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="D14" s="5" t="n">
         <v>24</v>
@@ -4502,10 +4532,10 @@
         <v>12</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="D15" s="5" t="n">
         <v>26</v>
@@ -4528,10 +4558,10 @@
         <v>13</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="D16" s="5" t="n">
         <v>24</v>
@@ -4554,10 +4584,10 @@
         <v>14</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="D17" s="5" t="n">
         <v>24</v>
@@ -4580,10 +4610,10 @@
         <v>15</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="D18" s="5" t="n">
         <v>27</v>
@@ -4606,10 +4636,10 @@
         <v>16</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D19" s="5" t="n">
         <v>25</v>
@@ -4632,10 +4662,10 @@
         <v>17</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="D20" s="5" t="n">
         <v>24</v>
@@ -4658,10 +4688,10 @@
         <v>18</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="D21" s="5" t="n">
         <v>27</v>
@@ -4684,10 +4714,10 @@
         <v>19</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="D22" s="5" t="n">
         <v>22</v>
@@ -4710,10 +4740,10 @@
         <v>20</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="D23" s="5" t="n">
         <v>27</v>
@@ -4736,10 +4766,10 @@
         <v>21</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="D24" s="5" t="n">
         <v>28</v>
@@ -4762,10 +4792,10 @@
         <v>22</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="D25" s="5" t="n">
         <v>27</v>
@@ -4788,10 +4818,10 @@
         <v>23</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="D26" s="5" t="n">
         <v>23</v>
@@ -4814,10 +4844,10 @@
         <v>24</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="D27" s="5" t="n">
         <v>27</v>
@@ -4840,10 +4870,10 @@
         <v>25</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="D28" s="5" t="n">
         <v>26</v>
@@ -4866,10 +4896,10 @@
         <v>26</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D29" s="5" t="n">
         <v>24</v>
@@ -4892,10 +4922,10 @@
         <v>27</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="D30" s="5" t="n">
         <v>25</v>
@@ -4918,10 +4948,10 @@
         <v>28</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="D31" s="5" t="n">
         <v>26</v>
@@ -4944,10 +4974,10 @@
         <v>29</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="D32" s="5" t="n">
         <v>21</v>
@@ -4970,10 +5000,10 @@
         <v>30</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D33" s="5" t="n">
         <v>28</v>
@@ -4996,10 +5026,10 @@
         <v>31</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="D34" s="5" t="n">
         <v>26</v>
@@ -5022,10 +5052,10 @@
         <v>32</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="D35" s="5" t="n">
         <v>26</v>
@@ -5045,7 +5075,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="8" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B36" s="9"/>
       <c r="C36" s="9"/>
@@ -5069,7 +5099,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="8" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B37" s="9"/>
       <c r="C37" s="9"/>
@@ -5096,7 +5126,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="13" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
     </row>
   </sheetData>
@@ -5128,33 +5158,33 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5162,7 +5192,7 @@
         <v>1</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C4" s="5" t="n">
         <v>19</v>
@@ -5184,7 +5214,7 @@
         <v>2</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="C5" s="5" t="n">
         <v>23</v>
@@ -5208,7 +5238,7 @@
         <v>3</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C6" s="5" t="n">
         <v>16</v>
@@ -5232,7 +5262,7 @@
         <v>4</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C7" s="5" t="n">
         <v>17</v>
@@ -5256,7 +5286,7 @@
         <v>5</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C8" s="5" t="n">
         <v>21</v>
@@ -5278,7 +5308,7 @@
         <v>6</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C9" s="5" t="n">
         <v>21</v>
@@ -5300,7 +5330,7 @@
         <v>7</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="C10" s="5" t="n">
         <v>22</v>
@@ -5322,7 +5352,7 @@
         <v>8</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C11" s="5" t="n">
         <v>21</v>
@@ -5346,7 +5376,7 @@
         <v>9</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="C12" s="5" t="n">
         <v>18</v>
@@ -5368,7 +5398,7 @@
         <v>10</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C13" s="5" t="n">
         <v>19</v>
@@ -5392,7 +5422,7 @@
         <v>11</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="C14" s="5" t="n">
         <v>19</v>
@@ -5414,7 +5444,7 @@
         <v>12</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="C15" s="5" t="n">
         <v>20</v>
@@ -5438,7 +5468,7 @@
         <v>13</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C16" s="5" t="n">
         <v>20</v>
@@ -5462,7 +5492,7 @@
         <v>14</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C17" s="5" t="n">
         <v>19</v>
@@ -5486,7 +5516,7 @@
         <v>15</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="C18" s="5" t="n">
         <v>22</v>
@@ -5510,7 +5540,7 @@
         <v>16</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="C19" s="5" t="n">
         <v>19</v>
@@ -5532,7 +5562,7 @@
         <v>17</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="C20" s="5" t="n">
         <v>18</v>
@@ -5556,7 +5586,7 @@
         <v>18</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C21" s="5" t="n">
         <v>19</v>
@@ -5578,7 +5608,7 @@
         <v>19</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C22" s="5" t="n">
         <v>18</v>
@@ -5602,7 +5632,7 @@
         <v>20</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="C23" s="5" t="n">
         <v>17</v>
@@ -5626,7 +5656,7 @@
         <v>21</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C24" s="5" t="n">
         <v>23</v>
@@ -5648,7 +5678,7 @@
         <v>22</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C25" s="5" t="n">
         <v>23</v>
@@ -5670,7 +5700,7 @@
         <v>23</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="C26" s="5" t="n">
         <v>19</v>
@@ -5692,7 +5722,7 @@
         <v>24</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C27" s="5" t="n">
         <v>19</v>
@@ -5714,7 +5744,7 @@
         <v>25</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="C28" s="5" t="n">
         <v>22</v>
@@ -5738,7 +5768,7 @@
         <v>26</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C29" s="5" t="n">
         <v>19</v>
@@ -5760,7 +5790,7 @@
         <v>27</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C30" s="5" t="n">
         <v>22</v>
@@ -5782,7 +5812,7 @@
         <v>28</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="C31" s="5" t="n">
         <v>19</v>
@@ -5804,7 +5834,7 @@
         <v>29</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C32" s="5" t="n">
         <v>18</v>
@@ -5828,7 +5858,7 @@
         <v>30</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C33" s="5" t="n">
         <v>20</v>
@@ -5850,7 +5880,7 @@
         <v>31</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="C34" s="5" t="n">
         <v>0</v>
@@ -5869,7 +5899,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="8" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B35" s="9"/>
       <c r="C35" s="10" t="n">
@@ -5893,7 +5923,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="8" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B36" s="9"/>
       <c r="C36" s="12" t="n">
@@ -5920,7 +5950,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="13" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="C37" s="16" t="n">
         <v>19.1</v>
@@ -5940,7 +5970,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="13" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="C38" s="16" t="n">
         <f aca="false">C36-C37</f>
@@ -5965,7 +5995,483 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="13" t="s">
-        <v>219</v>
+        <v>220</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:H22"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="6" style="0" width="16"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="3" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="D4" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="E4" s="6" t="n">
+        <v>28.3</v>
+      </c>
+      <c r="F4" s="7" t="n">
+        <v>1464680</v>
+      </c>
+      <c r="G4" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" s="7" t="n">
+        <v>1609905</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="C5" s="2"/>
+      <c r="D5" s="5" t="n">
+        <v>14</v>
+      </c>
+      <c r="E5" s="6" t="n">
+        <v>24.6</v>
+      </c>
+      <c r="F5" s="7" t="n">
+        <v>1125782</v>
+      </c>
+      <c r="G5" s="7" t="n">
+        <v>392288</v>
+      </c>
+      <c r="H5" s="7" t="n">
+        <v>1598069</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="D6" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="E6" s="6" t="n">
+        <v>27</v>
+      </c>
+      <c r="F6" s="7" t="n">
+        <v>1498709</v>
+      </c>
+      <c r="G6" s="7" t="n">
+        <v>7774</v>
+      </c>
+      <c r="H6" s="7" t="n">
+        <v>1572562</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="D7" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="E7" s="6" t="n">
+        <v>28.1</v>
+      </c>
+      <c r="F7" s="7" t="n">
+        <v>1428691</v>
+      </c>
+      <c r="G7" s="7" t="n">
+        <v>102055</v>
+      </c>
+      <c r="H7" s="7" t="n">
+        <v>1530746</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C8" s="2"/>
+      <c r="D8" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="E8" s="6" t="n">
+        <v>26.8</v>
+      </c>
+      <c r="F8" s="7" t="n">
+        <v>1438629</v>
+      </c>
+      <c r="G8" s="7" t="n">
+        <v>69420</v>
+      </c>
+      <c r="H8" s="7" t="n">
+        <v>1508049</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="D9" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="E9" s="6" t="n">
+        <v>29.3</v>
+      </c>
+      <c r="F9" s="7" t="n">
+        <v>1402693</v>
+      </c>
+      <c r="G9" s="7" t="n">
+        <v>103927</v>
+      </c>
+      <c r="H9" s="7" t="n">
+        <v>1506620</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>224</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="D10" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="E10" s="6" t="n">
+        <v>29.6</v>
+      </c>
+      <c r="F10" s="7" t="n">
+        <v>1402678</v>
+      </c>
+      <c r="G10" s="7" t="n">
+        <v>102257</v>
+      </c>
+      <c r="H10" s="7" t="n">
+        <v>1504935</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C11" s="2"/>
+      <c r="D11" s="5" t="n">
+        <v>16</v>
+      </c>
+      <c r="E11" s="6" t="n">
+        <v>28.3</v>
+      </c>
+      <c r="F11" s="7" t="n">
+        <v>1271683</v>
+      </c>
+      <c r="G11" s="7" t="n">
+        <v>219447</v>
+      </c>
+      <c r="H11" s="7" t="n">
+        <v>1491130</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="C12" s="2"/>
+      <c r="D12" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="E12" s="6" t="n">
+        <v>27.2</v>
+      </c>
+      <c r="F12" s="7" t="n">
+        <v>1312314</v>
+      </c>
+      <c r="G12" s="7" t="n">
+        <v>174720</v>
+      </c>
+      <c r="H12" s="7" t="n">
+        <v>1487034</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="C13" s="2"/>
+      <c r="D13" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="E13" s="6" t="n">
+        <v>27.6</v>
+      </c>
+      <c r="F13" s="7" t="n">
+        <v>1330240</v>
+      </c>
+      <c r="G13" s="7" t="n">
+        <v>149387</v>
+      </c>
+      <c r="H13" s="7" t="n">
+        <v>1479627</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="C14" s="2"/>
+      <c r="D14" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="E14" s="6" t="n">
+        <v>26.6</v>
+      </c>
+      <c r="F14" s="7" t="n">
+        <v>1040513</v>
+      </c>
+      <c r="G14" s="7" t="n">
+        <v>252240</v>
+      </c>
+      <c r="H14" s="7" t="n">
+        <v>1292753</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="D15" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="E15" s="6" t="n">
+        <v>26.7</v>
+      </c>
+      <c r="F15" s="7" t="n">
+        <v>1091805</v>
+      </c>
+      <c r="G15" s="7" t="n">
+        <v>195813</v>
+      </c>
+      <c r="H15" s="7" t="n">
+        <v>1287618</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="C16" s="2"/>
+      <c r="D16" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="E16" s="6" t="n">
+        <v>25.2</v>
+      </c>
+      <c r="F16" s="7" t="n">
+        <v>1091432</v>
+      </c>
+      <c r="G16" s="7" t="n">
+        <v>144450</v>
+      </c>
+      <c r="H16" s="7" t="n">
+        <v>1235882</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="B17" s="9"/>
+      <c r="C17" s="9"/>
+      <c r="D17" s="10" t="n">
+        <f aca="false">SUM(D4:D16)</f>
+        <v>162</v>
+      </c>
+      <c r="E17" s="9"/>
+      <c r="F17" s="11" t="n">
+        <f aca="false">SUM(F4:F16)</f>
+        <v>16899849</v>
+      </c>
+      <c r="G17" s="11" t="n">
+        <f aca="false">SUM(G4:G16)</f>
+        <v>1913778</v>
+      </c>
+      <c r="H17" s="11" t="n">
+        <f aca="false">SUM(H4:H16)</f>
+        <v>19104930</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="B18" s="9"/>
+      <c r="C18" s="9"/>
+      <c r="D18" s="12" t="n">
+        <f aca="false">AVERAGE(D4:D16)</f>
+        <v>12.4615384615385</v>
+      </c>
+      <c r="E18" s="12" t="n">
+        <f aca="false">AVERAGE(E4:E16)</f>
+        <v>27.3307692307692</v>
+      </c>
+      <c r="F18" s="11" t="n">
+        <f aca="false">AVERAGE(F4:F16)</f>
+        <v>1299988.38461538</v>
+      </c>
+      <c r="G18" s="11" t="n">
+        <f aca="false">AVERAGE(G4:G16)</f>
+        <v>147213.692307692</v>
+      </c>
+      <c r="H18" s="11" t="n">
+        <f aca="false">AVERAGE(H4:H16)</f>
+        <v>1469610</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="13" t="s">
+        <v>71</v>
+      </c>
+      <c r="D19" s="14" t="n">
+        <v>162</v>
+      </c>
+      <c r="F19" s="15" t="n">
+        <v>16899849</v>
+      </c>
+      <c r="G19" s="15" t="n">
+        <v>1913778</v>
+      </c>
+      <c r="H19" s="15" t="n">
+        <v>19104930</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="13" t="s">
+        <v>72</v>
+      </c>
+      <c r="D20" s="14" t="n">
+        <f aca="false">D17-D19</f>
+        <v>0</v>
+      </c>
+      <c r="F20" s="15" t="n">
+        <f aca="false">F17-F19</f>
+        <v>0</v>
+      </c>
+      <c r="G20" s="15" t="n">
+        <f aca="false">G17-G19</f>
+        <v>0</v>
+      </c>
+      <c r="H20" s="15" t="n">
+        <f aca="false">H17-H19</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="13" t="s">
+        <v>227</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add WNBA 2026 cash tab to Spotrac payroll workbook
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PFAktiXyafs53JJMEMzshM
</commit_message>
<xml_diff>
--- a/reports/Spotrac team payrolls.xlsx
+++ b/reports/Spotrac team payrolls.xlsx
@@ -14,7 +14,8 @@
     <sheet name="MLB" sheetId="4" state="visible" r:id="rId6"/>
     <sheet name="NHL" sheetId="5" state="visible" r:id="rId7"/>
     <sheet name="MLS" sheetId="6" state="visible" r:id="rId8"/>
-    <sheet name="WNBA" sheetId="7" state="visible" r:id="rId9"/>
+    <sheet name="WNBA 2025" sheetId="7" state="visible" r:id="rId9"/>
+    <sheet name="WNBA 2026" sheetId="8" state="visible" r:id="rId10"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -26,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="392" uniqueCount="228">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="423" uniqueCount="232">
   <si>
     <t xml:space="preserve">Spotrac team payroll tables transcribed from five screenshots supplied by the user (transcribed Oct 21, 2026).</t>
   </si>
@@ -46,7 +47,10 @@
     <t xml:space="preserve">NHL | Spotrac NHL cash tracker | Not shown; records match 2025-26 | Cash paid: Active + Dead + other. Screenshot had no totals row; totals here are SUM formulas.</t>
   </si>
   <si>
-    <t xml:space="preserve">WNBA | Spotrac WNBA cash tracker | 2025 (shown in screenshot) | Cash paid: Active + Dead + other</t>
+    <t xml:space="preserve">WNBA 2025 | Spotrac WNBA cash tracker | 2025 (shown in screenshot) | Cash paid: Active + Dead + other; 13 teams, cap $1,507,100</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WNBA 2026 | Spotrac WNBA cash tracker | 2026 (shown in screenshot) | Cash paid: Active + Dead + other; 15 teams, cap $7.0M under the 2026 CBA</t>
   </si>
   <si>
     <t xml:space="preserve">MLS | Spotrac MLS cap tracker | Not shown; likely 2026 | Cap allocation (not cash): Total Allocation = Senior + Supplemental + Dead. Row 31 'MLS' is league-held dead money.</t>
@@ -710,6 +714,15 @@
   </si>
   <si>
     <t xml:space="preserve">Spotrac's Record column showed only icons (star = playoff team, trophy = champion); those are written as text here.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WNBA 2026 team cash payroll (Spotrac)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spotrac's Record column was blank ('-') for every team in this screenshot.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">15 teams in 2026 after Toronto (TOR) and Portland (POR) expansion; 2026 salary cap $7.0M per team under the new CBA.</t>
   </si>
 </sst>
 </file>
@@ -1160,7 +1173,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:A16"/>
+  <dimension ref="A1:A17"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="150"/>
@@ -1210,12 +1223,12 @@
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="1"/>
+      <c r="A10" s="1" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="2" t="s">
-        <v>8</v>
-      </c>
+      <c r="A11" s="2"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
@@ -1240,6 +1253,11 @@
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
         <v>13</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="2" t="s">
+        <v>14</v>
       </c>
     </row>
   </sheetData>
@@ -1271,33 +1289,33 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1305,10 +1323,10 @@
         <v>1</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D4" s="5" t="n">
         <v>53</v>
@@ -1331,10 +1349,10 @@
         <v>2</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D5" s="5" t="n">
         <v>53</v>
@@ -1357,10 +1375,10 @@
         <v>3</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D6" s="5" t="n">
         <v>54</v>
@@ -1383,10 +1401,10 @@
         <v>4</v>
       </c>
       <c r="B7" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C7" s="2" t="s">
         <v>29</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>28</v>
       </c>
       <c r="D7" s="5" t="n">
         <v>52</v>
@@ -1409,10 +1427,10 @@
         <v>5</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D8" s="5" t="n">
         <v>52</v>
@@ -1435,10 +1453,10 @@
         <v>6</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D9" s="5" t="n">
         <v>52</v>
@@ -1461,10 +1479,10 @@
         <v>7</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D10" s="5" t="n">
         <v>52</v>
@@ -1487,10 +1505,10 @@
         <v>8</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D11" s="5" t="n">
         <v>53</v>
@@ -1513,10 +1531,10 @@
         <v>9</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D12" s="5" t="n">
         <v>53</v>
@@ -1539,10 +1557,10 @@
         <v>10</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D13" s="5" t="n">
         <v>53</v>
@@ -1565,10 +1583,10 @@
         <v>11</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D14" s="5" t="n">
         <v>52</v>
@@ -1591,10 +1609,10 @@
         <v>12</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D15" s="5" t="n">
         <v>53</v>
@@ -1617,10 +1635,10 @@
         <v>13</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D16" s="5" t="n">
         <v>51</v>
@@ -1643,10 +1661,10 @@
         <v>14</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D17" s="5" t="n">
         <v>53</v>
@@ -1669,10 +1687,10 @@
         <v>15</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D18" s="5" t="n">
         <v>52</v>
@@ -1695,10 +1713,10 @@
         <v>16</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D19" s="5" t="n">
         <v>54</v>
@@ -1721,10 +1739,10 @@
         <v>17</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D20" s="5" t="n">
         <v>53</v>
@@ -1747,10 +1765,10 @@
         <v>18</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D21" s="5" t="n">
         <v>53</v>
@@ -1773,10 +1791,10 @@
         <v>19</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D22" s="5" t="n">
         <v>52</v>
@@ -1799,10 +1817,10 @@
         <v>20</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D23" s="5" t="n">
         <v>52</v>
@@ -1825,10 +1843,10 @@
         <v>21</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D24" s="5" t="n">
         <v>53</v>
@@ -1851,10 +1869,10 @@
         <v>22</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D25" s="5" t="n">
         <v>53</v>
@@ -1877,10 +1895,10 @@
         <v>23</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D26" s="5" t="n">
         <v>53</v>
@@ -1903,10 +1921,10 @@
         <v>24</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D27" s="5" t="n">
         <v>52</v>
@@ -1929,10 +1947,10 @@
         <v>25</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D28" s="5" t="n">
         <v>53</v>
@@ -1955,10 +1973,10 @@
         <v>26</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D29" s="5" t="n">
         <v>53</v>
@@ -1981,10 +1999,10 @@
         <v>27</v>
       </c>
       <c r="B30" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C30" s="2" t="s">
         <v>63</v>
-      </c>
-      <c r="C30" s="2" t="s">
-        <v>62</v>
       </c>
       <c r="D30" s="5" t="n">
         <v>52</v>
@@ -2007,10 +2025,10 @@
         <v>28</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D31" s="5" t="n">
         <v>53</v>
@@ -2033,10 +2051,10 @@
         <v>29</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D32" s="5" t="n">
         <v>52</v>
@@ -2059,10 +2077,10 @@
         <v>30</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D33" s="5" t="n">
         <v>52</v>
@@ -2085,10 +2103,10 @@
         <v>31</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D34" s="5" t="n">
         <v>53</v>
@@ -2111,10 +2129,10 @@
         <v>32</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D35" s="5" t="n">
         <v>53</v>
@@ -2134,7 +2152,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="8" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B36" s="9"/>
       <c r="C36" s="9"/>
@@ -2158,7 +2176,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="8" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B37" s="9"/>
       <c r="C37" s="9"/>
@@ -2185,7 +2203,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="13" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D38" s="14" t="n">
         <v>1684</v>
@@ -2202,7 +2220,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="13" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D39" s="14" t="n">
         <f aca="false">D36-D38</f>
@@ -2250,36 +2268,36 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="I3" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2287,10 +2305,10 @@
         <v>28</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D4" s="5" t="n">
         <v>15</v>
@@ -2316,10 +2334,10 @@
         <v>15</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D5" s="5" t="n">
         <v>15</v>
@@ -2345,10 +2363,10 @@
         <v>1</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D6" s="5" t="n">
         <v>15</v>
@@ -2374,10 +2392,10 @@
         <v>2</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D7" s="5" t="n">
         <v>15</v>
@@ -2403,10 +2421,10 @@
         <v>8</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D8" s="5" t="n">
         <v>15</v>
@@ -2432,10 +2450,10 @@
         <v>23</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D9" s="5" t="n">
         <v>15</v>
@@ -2461,10 +2479,10 @@
         <v>26</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D10" s="5" t="n">
         <v>15</v>
@@ -2490,10 +2508,10 @@
         <v>10</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D11" s="5" t="n">
         <v>15</v>
@@ -2519,10 +2537,10 @@
         <v>4</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D12" s="5" t="n">
         <v>15</v>
@@ -2548,10 +2566,10 @@
         <v>16</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D13" s="5" t="n">
         <v>15</v>
@@ -2577,10 +2595,10 @@
         <v>5</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D14" s="5" t="n">
         <v>15</v>
@@ -2606,10 +2624,10 @@
         <v>22</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D15" s="5" t="n">
         <v>15</v>
@@ -2635,10 +2653,10 @@
         <v>29</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D16" s="5" t="n">
         <v>15</v>
@@ -2664,10 +2682,10 @@
         <v>7</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D17" s="5" t="n">
         <v>15</v>
@@ -2693,10 +2711,10 @@
         <v>25</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D18" s="5" t="n">
         <v>15</v>
@@ -2722,10 +2740,10 @@
         <v>6</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D19" s="5" t="n">
         <v>15</v>
@@ -2751,10 +2769,10 @@
         <v>11</v>
       </c>
       <c r="B20" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="C20" s="2" t="s">
         <v>96</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>95</v>
       </c>
       <c r="D20" s="5" t="n">
         <v>15</v>
@@ -2780,10 +2798,10 @@
         <v>14</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D21" s="5" t="n">
         <v>15</v>
@@ -2809,10 +2827,10 @@
         <v>13</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D22" s="5" t="n">
         <v>15</v>
@@ -2838,10 +2856,10 @@
         <v>19</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D23" s="5" t="n">
         <v>15</v>
@@ -2867,10 +2885,10 @@
         <v>24</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D24" s="5" t="n">
         <v>15</v>
@@ -2896,10 +2914,10 @@
         <v>3</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D25" s="5" t="n">
         <v>15</v>
@@ -2925,10 +2943,10 @@
         <v>20</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D26" s="5" t="n">
         <v>15</v>
@@ -2954,10 +2972,10 @@
         <v>27</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D27" s="5" t="n">
         <v>15</v>
@@ -2983,10 +3001,10 @@
         <v>12</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D28" s="5" t="n">
         <v>15</v>
@@ -3012,10 +3030,10 @@
         <v>17</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D29" s="5" t="n">
         <v>15</v>
@@ -3041,10 +3059,10 @@
         <v>9</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D30" s="5" t="n">
         <v>15</v>
@@ -3070,10 +3088,10 @@
         <v>18</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D31" s="5" t="n">
         <v>15</v>
@@ -3099,10 +3117,10 @@
         <v>30</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D32" s="5" t="n">
         <v>15</v>
@@ -3128,10 +3146,10 @@
         <v>21</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D33" s="5" t="n">
         <v>15</v>
@@ -3154,7 +3172,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="8" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B34" s="9"/>
       <c r="C34" s="9"/>
@@ -3182,7 +3200,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="8" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B35" s="9"/>
       <c r="C35" s="9"/>
@@ -3213,7 +3231,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="13" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D36" s="14" t="n">
         <v>450</v>
@@ -3233,7 +3251,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="13" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D37" s="14" t="n">
         <f aca="false">D34-D36</f>
@@ -3285,33 +3303,33 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3319,10 +3337,10 @@
         <v>1</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D4" s="5" t="n">
         <v>28</v>
@@ -3345,10 +3363,10 @@
         <v>2</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D5" s="5" t="n">
         <v>27</v>
@@ -3371,10 +3389,10 @@
         <v>3</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D6" s="5" t="n">
         <v>28</v>
@@ -3397,10 +3415,10 @@
         <v>4</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D7" s="5" t="n">
         <v>27</v>
@@ -3423,10 +3441,10 @@
         <v>5</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D8" s="5" t="n">
         <v>28</v>
@@ -3449,10 +3467,10 @@
         <v>6</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="D9" s="5" t="n">
         <v>28</v>
@@ -3475,10 +3493,10 @@
         <v>7</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D10" s="5" t="n">
         <v>32</v>
@@ -3501,10 +3519,10 @@
         <v>8</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="D11" s="5" t="n">
         <v>28</v>
@@ -3527,10 +3545,10 @@
         <v>9</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D12" s="5" t="n">
         <v>28</v>
@@ -3553,10 +3571,10 @@
         <v>10</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D13" s="5" t="n">
         <v>28</v>
@@ -3579,10 +3597,10 @@
         <v>11</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D14" s="5" t="n">
         <v>28</v>
@@ -3605,10 +3623,10 @@
         <v>12</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D15" s="5" t="n">
         <v>28</v>
@@ -3631,10 +3649,10 @@
         <v>13</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D16" s="5" t="n">
         <v>28</v>
@@ -3657,10 +3675,10 @@
         <v>14</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D17" s="5" t="n">
         <v>28</v>
@@ -3683,10 +3701,10 @@
         <v>15</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D18" s="5" t="n">
         <v>28</v>
@@ -3709,10 +3727,10 @@
         <v>16</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D19" s="5" t="n">
         <v>28</v>
@@ -3735,10 +3753,10 @@
         <v>17</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="D20" s="5" t="n">
         <v>28</v>
@@ -3761,10 +3779,10 @@
         <v>18</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D21" s="5" t="n">
         <v>28</v>
@@ -3787,10 +3805,10 @@
         <v>19</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="D22" s="5" t="n">
         <v>28</v>
@@ -3813,10 +3831,10 @@
         <v>20</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D23" s="5" t="n">
         <v>28</v>
@@ -3839,10 +3857,10 @@
         <v>21</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="D24" s="5" t="n">
         <v>28</v>
@@ -3865,10 +3883,10 @@
         <v>22</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D25" s="5" t="n">
         <v>28</v>
@@ -3891,10 +3909,10 @@
         <v>23</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D26" s="5" t="n">
         <v>28</v>
@@ -3917,10 +3935,10 @@
         <v>24</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D27" s="5" t="n">
         <v>28</v>
@@ -3943,10 +3961,10 @@
         <v>25</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="D28" s="5" t="n">
         <v>28</v>
@@ -3969,10 +3987,10 @@
         <v>26</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="D29" s="5" t="n">
         <v>28</v>
@@ -3995,10 +4013,10 @@
         <v>27</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D30" s="5" t="n">
         <v>31</v>
@@ -4021,10 +4039,10 @@
         <v>28</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="D31" s="5" t="n">
         <v>28</v>
@@ -4047,10 +4065,10 @@
         <v>29</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="D32" s="5" t="n">
         <v>28</v>
@@ -4073,10 +4091,10 @@
         <v>30</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D33" s="5" t="n">
         <v>28</v>
@@ -4096,7 +4114,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="8" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B34" s="9"/>
       <c r="C34" s="9"/>
@@ -4120,7 +4138,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="8" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B35" s="9"/>
       <c r="C35" s="9"/>
@@ -4147,7 +4165,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="13" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D36" s="14" t="n">
         <v>845</v>
@@ -4164,7 +4182,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="13" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D37" s="14" t="n">
         <f aca="false">D34-D36</f>
@@ -4212,33 +4230,33 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4246,10 +4264,10 @@
         <v>1</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="D4" s="5" t="n">
         <v>23</v>
@@ -4272,10 +4290,10 @@
         <v>2</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D5" s="5" t="n">
         <v>27</v>
@@ -4298,10 +4316,10 @@
         <v>3</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D6" s="5" t="n">
         <v>24</v>
@@ -4324,10 +4342,10 @@
         <v>4</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="D7" s="5" t="n">
         <v>25</v>
@@ -4350,10 +4368,10 @@
         <v>5</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="D8" s="5" t="n">
         <v>22</v>
@@ -4376,10 +4394,10 @@
         <v>6</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="D9" s="5" t="n">
         <v>26</v>
@@ -4402,10 +4420,10 @@
         <v>7</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="D10" s="5" t="n">
         <v>23</v>
@@ -4428,10 +4446,10 @@
         <v>8</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="D11" s="5" t="n">
         <v>26</v>
@@ -4454,10 +4472,10 @@
         <v>9</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="D12" s="5" t="n">
         <v>26</v>
@@ -4480,10 +4498,10 @@
         <v>10</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D13" s="5" t="n">
         <v>25</v>
@@ -4506,10 +4524,10 @@
         <v>11</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="D14" s="5" t="n">
         <v>24</v>
@@ -4532,10 +4550,10 @@
         <v>12</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="D15" s="5" t="n">
         <v>26</v>
@@ -4558,10 +4576,10 @@
         <v>13</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="D16" s="5" t="n">
         <v>24</v>
@@ -4584,10 +4602,10 @@
         <v>14</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="D17" s="5" t="n">
         <v>24</v>
@@ -4610,10 +4628,10 @@
         <v>15</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D18" s="5" t="n">
         <v>27</v>
@@ -4636,10 +4654,10 @@
         <v>16</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="D19" s="5" t="n">
         <v>25</v>
@@ -4662,10 +4680,10 @@
         <v>17</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="D20" s="5" t="n">
         <v>24</v>
@@ -4688,10 +4706,10 @@
         <v>18</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="D21" s="5" t="n">
         <v>27</v>
@@ -4714,10 +4732,10 @@
         <v>19</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="D22" s="5" t="n">
         <v>22</v>
@@ -4740,10 +4758,10 @@
         <v>20</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="D23" s="5" t="n">
         <v>27</v>
@@ -4766,10 +4784,10 @@
         <v>21</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="D24" s="5" t="n">
         <v>28</v>
@@ -4792,10 +4810,10 @@
         <v>22</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="D25" s="5" t="n">
         <v>27</v>
@@ -4818,10 +4836,10 @@
         <v>23</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="D26" s="5" t="n">
         <v>23</v>
@@ -4844,10 +4862,10 @@
         <v>24</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="D27" s="5" t="n">
         <v>27</v>
@@ -4870,10 +4888,10 @@
         <v>25</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="D28" s="5" t="n">
         <v>26</v>
@@ -4896,10 +4914,10 @@
         <v>26</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="D29" s="5" t="n">
         <v>24</v>
@@ -4922,10 +4940,10 @@
         <v>27</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="D30" s="5" t="n">
         <v>25</v>
@@ -4948,10 +4966,10 @@
         <v>28</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="D31" s="5" t="n">
         <v>26</v>
@@ -4974,10 +4992,10 @@
         <v>29</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="D32" s="5" t="n">
         <v>21</v>
@@ -5000,10 +5018,10 @@
         <v>30</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="D33" s="5" t="n">
         <v>28</v>
@@ -5026,10 +5044,10 @@
         <v>31</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="D34" s="5" t="n">
         <v>26</v>
@@ -5052,10 +5070,10 @@
         <v>32</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="D35" s="5" t="n">
         <v>26</v>
@@ -5075,7 +5093,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="8" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B36" s="9"/>
       <c r="C36" s="9"/>
@@ -5099,7 +5117,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="8" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B37" s="9"/>
       <c r="C37" s="9"/>
@@ -5126,7 +5144,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="13" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
     </row>
   </sheetData>
@@ -5158,33 +5176,33 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5192,7 +5210,7 @@
         <v>1</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C4" s="5" t="n">
         <v>19</v>
@@ -5214,7 +5232,7 @@
         <v>2</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="C5" s="5" t="n">
         <v>23</v>
@@ -5238,7 +5256,7 @@
         <v>3</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C6" s="5" t="n">
         <v>16</v>
@@ -5262,7 +5280,7 @@
         <v>4</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C7" s="5" t="n">
         <v>17</v>
@@ -5286,7 +5304,7 @@
         <v>5</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C8" s="5" t="n">
         <v>21</v>
@@ -5308,7 +5326,7 @@
         <v>6</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C9" s="5" t="n">
         <v>21</v>
@@ -5330,7 +5348,7 @@
         <v>7</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="C10" s="5" t="n">
         <v>22</v>
@@ -5352,7 +5370,7 @@
         <v>8</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C11" s="5" t="n">
         <v>21</v>
@@ -5376,7 +5394,7 @@
         <v>9</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="C12" s="5" t="n">
         <v>18</v>
@@ -5398,7 +5416,7 @@
         <v>10</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C13" s="5" t="n">
         <v>19</v>
@@ -5422,7 +5440,7 @@
         <v>11</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="C14" s="5" t="n">
         <v>19</v>
@@ -5444,7 +5462,7 @@
         <v>12</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="C15" s="5" t="n">
         <v>20</v>
@@ -5468,7 +5486,7 @@
         <v>13</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C16" s="5" t="n">
         <v>20</v>
@@ -5492,7 +5510,7 @@
         <v>14</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C17" s="5" t="n">
         <v>19</v>
@@ -5516,7 +5534,7 @@
         <v>15</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="C18" s="5" t="n">
         <v>22</v>
@@ -5540,7 +5558,7 @@
         <v>16</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="C19" s="5" t="n">
         <v>19</v>
@@ -5562,7 +5580,7 @@
         <v>17</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="C20" s="5" t="n">
         <v>18</v>
@@ -5586,7 +5604,7 @@
         <v>18</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C21" s="5" t="n">
         <v>19</v>
@@ -5608,7 +5626,7 @@
         <v>19</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C22" s="5" t="n">
         <v>18</v>
@@ -5632,7 +5650,7 @@
         <v>20</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="C23" s="5" t="n">
         <v>17</v>
@@ -5656,7 +5674,7 @@
         <v>21</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C24" s="5" t="n">
         <v>23</v>
@@ -5678,7 +5696,7 @@
         <v>22</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C25" s="5" t="n">
         <v>23</v>
@@ -5700,7 +5718,7 @@
         <v>23</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="C26" s="5" t="n">
         <v>19</v>
@@ -5722,7 +5740,7 @@
         <v>24</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C27" s="5" t="n">
         <v>19</v>
@@ -5744,7 +5762,7 @@
         <v>25</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C28" s="5" t="n">
         <v>22</v>
@@ -5768,7 +5786,7 @@
         <v>26</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="C29" s="5" t="n">
         <v>19</v>
@@ -5790,7 +5808,7 @@
         <v>27</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C30" s="5" t="n">
         <v>22</v>
@@ -5812,7 +5830,7 @@
         <v>28</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="C31" s="5" t="n">
         <v>19</v>
@@ -5834,7 +5852,7 @@
         <v>29</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="C32" s="5" t="n">
         <v>18</v>
@@ -5858,7 +5876,7 @@
         <v>30</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C33" s="5" t="n">
         <v>20</v>
@@ -5880,7 +5898,7 @@
         <v>31</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="C34" s="5" t="n">
         <v>0</v>
@@ -5899,7 +5917,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="8" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B35" s="9"/>
       <c r="C35" s="10" t="n">
@@ -5923,7 +5941,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="8" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B36" s="9"/>
       <c r="C36" s="12" t="n">
@@ -5950,7 +5968,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="13" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="C37" s="16" t="n">
         <v>19.1</v>
@@ -5970,7 +5988,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="13" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="C38" s="16" t="n">
         <f aca="false">C36-C37</f>
@@ -5995,7 +6013,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="13" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
   </sheetData>
@@ -6027,33 +6045,33 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6061,10 +6079,10 @@
         <v>1</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="D4" s="5" t="n">
         <v>12</v>
@@ -6087,7 +6105,7 @@
         <v>2</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C5" s="2"/>
       <c r="D5" s="5" t="n">
@@ -6111,10 +6129,10 @@
         <v>3</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="D6" s="5" t="n">
         <v>12</v>
@@ -6137,10 +6155,10 @@
         <v>4</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="D7" s="5" t="n">
         <v>11</v>
@@ -6163,7 +6181,7 @@
         <v>5</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C8" s="2"/>
       <c r="D8" s="5" t="n">
@@ -6187,10 +6205,10 @@
         <v>6</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="D9" s="5" t="n">
         <v>12</v>
@@ -6213,10 +6231,10 @@
         <v>7</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="D10" s="5" t="n">
         <v>12</v>
@@ -6239,7 +6257,7 @@
         <v>8</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C11" s="2"/>
       <c r="D11" s="5" t="n">
@@ -6263,7 +6281,7 @@
         <v>9</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="C12" s="2"/>
       <c r="D12" s="5" t="n">
@@ -6287,7 +6305,7 @@
         <v>10</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C13" s="2"/>
       <c r="D13" s="5" t="n">
@@ -6311,7 +6329,7 @@
         <v>11</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="C14" s="2"/>
       <c r="D14" s="5" t="n">
@@ -6335,10 +6353,10 @@
         <v>12</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="D15" s="5" t="n">
         <v>13</v>
@@ -6361,7 +6379,7 @@
         <v>13</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C16" s="2"/>
       <c r="D16" s="5" t="n">
@@ -6382,7 +6400,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="8" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B17" s="9"/>
       <c r="C17" s="9"/>
@@ -6406,7 +6424,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="8" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B18" s="9"/>
       <c r="C18" s="9"/>
@@ -6433,7 +6451,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="13" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D19" s="14" t="n">
         <v>162</v>
@@ -6450,7 +6468,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="13" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D20" s="14" t="n">
         <f aca="false">D17-D19</f>
@@ -6471,7 +6489,524 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="13" t="s">
+        <v>228</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:H25"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="6" style="0" width="16"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="3" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="2" t="s">
         <v>227</v>
+      </c>
+      <c r="C4" s="2"/>
+      <c r="D4" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="E4" s="6" t="n">
+        <v>27.8</v>
+      </c>
+      <c r="F4" s="7" t="n">
+        <v>6386195</v>
+      </c>
+      <c r="G4" s="7" t="n">
+        <v>298536</v>
+      </c>
+      <c r="H4" s="7" t="n">
+        <v>7134731</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="C5" s="2"/>
+      <c r="D5" s="5" t="n">
+        <v>14</v>
+      </c>
+      <c r="E5" s="6" t="n">
+        <v>28.3</v>
+      </c>
+      <c r="F5" s="7" t="n">
+        <v>6992195</v>
+      </c>
+      <c r="G5" s="7" t="n">
+        <v>139878</v>
+      </c>
+      <c r="H5" s="7" t="n">
+        <v>7132073</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C6" s="2"/>
+      <c r="D6" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="E6" s="6" t="n">
+        <v>29.5</v>
+      </c>
+      <c r="F6" s="7" t="n">
+        <v>6844199</v>
+      </c>
+      <c r="G6" s="7" t="n">
+        <v>226098</v>
+      </c>
+      <c r="H6" s="7" t="n">
+        <v>7070297</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C7" s="2"/>
+      <c r="D7" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="E7" s="6" t="n">
+        <v>28.2</v>
+      </c>
+      <c r="F7" s="7" t="n">
+        <v>6814604</v>
+      </c>
+      <c r="G7" s="7" t="n">
+        <v>248415</v>
+      </c>
+      <c r="H7" s="7" t="n">
+        <v>7063019</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C8" s="2"/>
+      <c r="D8" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="E8" s="6" t="n">
+        <v>27.2</v>
+      </c>
+      <c r="F8" s="7" t="n">
+        <v>7022675</v>
+      </c>
+      <c r="G8" s="7" t="n">
+        <v>36098</v>
+      </c>
+      <c r="H8" s="7" t="n">
+        <v>7058773</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="C9" s="2"/>
+      <c r="D9" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="E9" s="6" t="n">
+        <v>28.5</v>
+      </c>
+      <c r="F9" s="7" t="n">
+        <v>5360855</v>
+      </c>
+      <c r="G9" s="7" t="n">
+        <v>860551</v>
+      </c>
+      <c r="H9" s="7" t="n">
+        <v>6991406</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C10" s="2"/>
+      <c r="D10" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="E10" s="6" t="n">
+        <v>27.9</v>
+      </c>
+      <c r="F10" s="7" t="n">
+        <v>6579603</v>
+      </c>
+      <c r="G10" s="7" t="n">
+        <v>284268</v>
+      </c>
+      <c r="H10" s="7" t="n">
+        <v>6863871</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="C11" s="2"/>
+      <c r="D11" s="5" t="n">
+        <v>14</v>
+      </c>
+      <c r="E11" s="6" t="n">
+        <v>28.3</v>
+      </c>
+      <c r="F11" s="7" t="n">
+        <v>6456810</v>
+      </c>
+      <c r="G11" s="7" t="n">
+        <v>347928</v>
+      </c>
+      <c r="H11" s="7" t="n">
+        <v>6804738</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C12" s="2"/>
+      <c r="D12" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="E12" s="6" t="n">
+        <v>27.5</v>
+      </c>
+      <c r="F12" s="7" t="n">
+        <v>6503057</v>
+      </c>
+      <c r="G12" s="7" t="n">
+        <v>144878</v>
+      </c>
+      <c r="H12" s="7" t="n">
+        <v>6647935</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="C13" s="2"/>
+      <c r="D13" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="E13" s="6" t="n">
+        <v>28.6</v>
+      </c>
+      <c r="F13" s="7" t="n">
+        <v>6491010</v>
+      </c>
+      <c r="G13" s="7" t="n">
+        <v>69086</v>
+      </c>
+      <c r="H13" s="7" t="n">
+        <v>6560096</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="C14" s="2"/>
+      <c r="D14" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="E14" s="6" t="n">
+        <v>28.3</v>
+      </c>
+      <c r="F14" s="7" t="n">
+        <v>5979034</v>
+      </c>
+      <c r="G14" s="7" t="n">
+        <v>564756</v>
+      </c>
+      <c r="H14" s="7" t="n">
+        <v>6543790</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="C15" s="2"/>
+      <c r="D15" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="E15" s="6" t="n">
+        <v>25.3</v>
+      </c>
+      <c r="F15" s="7" t="n">
+        <v>5977390</v>
+      </c>
+      <c r="G15" s="7" t="n">
+        <v>346647</v>
+      </c>
+      <c r="H15" s="7" t="n">
+        <v>6324037</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="C16" s="2"/>
+      <c r="D16" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="E16" s="6" t="n">
+        <v>24.8</v>
+      </c>
+      <c r="F16" s="7" t="n">
+        <v>5606834</v>
+      </c>
+      <c r="G16" s="7" t="n">
+        <v>360896</v>
+      </c>
+      <c r="H16" s="7" t="n">
+        <v>5967730</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="5" t="n">
+        <v>14</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C17" s="2"/>
+      <c r="D17" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="E17" s="6" t="n">
+        <v>23.9</v>
+      </c>
+      <c r="F17" s="7" t="n">
+        <v>5231898</v>
+      </c>
+      <c r="G17" s="7" t="n">
+        <v>331463</v>
+      </c>
+      <c r="H17" s="7" t="n">
+        <v>5563361</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="C18" s="2"/>
+      <c r="D18" s="5" t="n">
+        <v>14</v>
+      </c>
+      <c r="E18" s="6" t="n">
+        <v>26</v>
+      </c>
+      <c r="F18" s="7" t="n">
+        <v>4672338</v>
+      </c>
+      <c r="G18" s="7" t="n">
+        <v>445163</v>
+      </c>
+      <c r="H18" s="7" t="n">
+        <v>5117501</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="B19" s="9"/>
+      <c r="C19" s="9"/>
+      <c r="D19" s="10" t="n">
+        <f aca="false">SUM(D4:D18)</f>
+        <v>189</v>
+      </c>
+      <c r="E19" s="9"/>
+      <c r="F19" s="11" t="n">
+        <f aca="false">SUM(F4:F18)</f>
+        <v>92918697</v>
+      </c>
+      <c r="G19" s="11" t="n">
+        <f aca="false">SUM(G4:G18)</f>
+        <v>4704661</v>
+      </c>
+      <c r="H19" s="11" t="n">
+        <f aca="false">SUM(H4:H18)</f>
+        <v>98843358</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="B20" s="9"/>
+      <c r="C20" s="9"/>
+      <c r="D20" s="12" t="n">
+        <f aca="false">AVERAGE(D4:D18)</f>
+        <v>12.6</v>
+      </c>
+      <c r="E20" s="12" t="n">
+        <f aca="false">AVERAGE(E4:E18)</f>
+        <v>27.34</v>
+      </c>
+      <c r="F20" s="11" t="n">
+        <f aca="false">AVERAGE(F4:F18)</f>
+        <v>6194579.8</v>
+      </c>
+      <c r="G20" s="11" t="n">
+        <f aca="false">AVERAGE(G4:G18)</f>
+        <v>313644.066666667</v>
+      </c>
+      <c r="H20" s="11" t="n">
+        <f aca="false">AVERAGE(H4:H18)</f>
+        <v>6589557.2</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="13" t="s">
+        <v>72</v>
+      </c>
+      <c r="D21" s="14" t="n">
+        <v>189</v>
+      </c>
+      <c r="F21" s="15" t="n">
+        <v>92918697</v>
+      </c>
+      <c r="G21" s="15" t="n">
+        <v>4704661</v>
+      </c>
+      <c r="H21" s="15" t="n">
+        <v>98843358</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="13" t="s">
+        <v>73</v>
+      </c>
+      <c r="D22" s="14" t="n">
+        <f aca="false">D19-D21</f>
+        <v>0</v>
+      </c>
+      <c r="F22" s="15" t="n">
+        <f aca="false">F19-F21</f>
+        <v>0</v>
+      </c>
+      <c r="G22" s="15" t="n">
+        <f aca="false">G19-G21</f>
+        <v>0</v>
+      </c>
+      <c r="H22" s="15" t="n">
+        <f aca="false">H19-H21</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="13" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="13" t="s">
+        <v>231</v>
       </c>
     </row>
   </sheetData>

</xml_diff>